<commit_message>
STM32 product added LPUART and Refman/ erratasheet outputs
</commit_message>
<xml_diff>
--- a/product_selector_out/STM32 Arm Cortex MPUs - diff.xlsx
+++ b/product_selector_out/STM32 Arm Cortex MPUs - diff.xlsx
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3456</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="6">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3251</v>
+        <v>3315</v>
       </c>
     </row>
     <row r="18">

</xml_diff>